<commit_message>
feature: push notification across cors
</commit_message>
<xml_diff>
--- a/Documents/Import/ProdLine.xlsx
+++ b/Documents/Import/ProdLine.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitLabSample\GitHub\JogetMVC\Documents\Import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2161F24B-19DA-40F1-9148-D434E0FD14C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9095669-C59F-4A31-9B11-9118B4448D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28935" yWindow="-7980" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FB316830-DCD3-473A-8A97-D2FCD8CA1E26}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{FB316830-DCD3-473A-8A97-D2FCD8CA1E26}"/>
   </bookViews>
   <sheets>
     <sheet name="Product" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="370">
   <si>
     <t>id</t>
   </si>
@@ -1139,6 +1139,18 @@
   </si>
   <si>
     <t>INNER JOIN [Product] ON [Product].ProductCode = Quotation.ProductCode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UPDATE Quotation SET LineId = 1 </t>
+  </si>
+  <si>
+    <t>UPDATE Quotation SET Quotation.LineName = Line.LineName</t>
+  </si>
+  <si>
+    <t>INNER JOIN Line ON Line.Id = Quotation.LineId</t>
+  </si>
+  <si>
+    <t>SELECT*  FROM Line</t>
   </si>
 </sst>
 </file>
@@ -5082,7 +5094,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C4A5B1E-4C60-4C18-91BB-188055C3917C}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.4">
@@ -5113,6 +5125,31 @@
     <row r="6" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>365</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A8" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A11" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>369</v>
       </c>
     </row>
   </sheetData>

</xml_diff>